<commit_message>
get weather with date arguments
</commit_message>
<xml_diff>
--- a/GET_WEATHER_RESULTS_TripId_1_Brasov.xlsx
+++ b/GET_WEATHER_RESULTS_TripId_1_Brasov.xlsx
@@ -31,13 +31,13 @@
     <x:t>1</x:t>
   </x:si>
   <x:si>
-    <x:t>-5.1°C</x:t>
-  </x:si>
-  <x:si>
-    <x:t>100%</x:t>
-  </x:si>
-  <x:si>
-    <x:t>The forecast for Brasov shows an average temperature of -5.1°C with a rain probability of 100%.</x:t>
+    <x:t>17.7</x:t>
+  </x:si>
+  <x:si>
+    <x:t>52%</x:t>
+  </x:si>
+  <x:si>
+    <x:t>The forecast for Brasov during 15 May 2026 - 20 July 2026 shows an average temperature of 17.7°C with a rain probability of 52%.</x:t>
   </x:si>
 </x:sst>
 </file>

</xml_diff>